<commit_message>
Added slides and updated test schedule
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -768,7 +768,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -886,6 +886,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5236,11 +5240,11 @@
       <c r="B5" s="29"/>
       <c r="C5" s="29"/>
       <c r="D5" s="29"/>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
       <c r="H5" s="13" t="s">
         <v>149</v>
       </c>
@@ -5256,11 +5260,11 @@
       </c>
       <c r="O5" s="17"/>
       <c r="P5" s="17"/>
-      <c r="Q5" s="30" t="s">
+      <c r="Q5" s="31" t="s">
         <v>151</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="31"/>
       <c r="T5" s="13" t="s">
         <v>152</v>
       </c>
@@ -5271,11 +5275,11 @@
       </c>
       <c r="X5" s="17"/>
       <c r="Y5" s="17"/>
-      <c r="Z5" s="17" t="s">
+      <c r="Z5" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="AA5" s="17"/>
-      <c r="AB5" s="17"/>
+      <c r="AA5" s="30"/>
+      <c r="AB5" s="30"/>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
@@ -5302,21 +5306,21 @@
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
-      <c r="Q6" s="30" t="s">
+      <c r="Q6" s="31" t="s">
         <v>158</v>
       </c>
-      <c r="R6" s="30"/>
-      <c r="S6" s="30"/>
+      <c r="R6" s="31"/>
+      <c r="S6" s="31"/>
       <c r="T6" s="13" t="s">
         <v>159</v>
       </c>
       <c r="U6" s="13"/>
       <c r="V6" s="13"/>
-      <c r="W6" s="31" t="s">
+      <c r="W6" s="32" t="s">
         <v>159</v>
       </c>
-      <c r="X6" s="31"/>
-      <c r="Y6" s="31"/>
+      <c r="X6" s="32"/>
+      <c r="Y6" s="32"/>
       <c r="Z6" s="17" t="s">
         <v>154</v>
       </c>
@@ -5348,11 +5352,11 @@
       </c>
       <c r="O7" s="17"/>
       <c r="P7" s="17"/>
-      <c r="Q7" s="30" t="s">
+      <c r="Q7" s="31" t="s">
         <v>163</v>
       </c>
-      <c r="R7" s="30"/>
-      <c r="S7" s="30"/>
+      <c r="R7" s="31"/>
+      <c r="S7" s="31"/>
       <c r="T7" s="13" t="s">
         <v>164</v>
       </c>

</xml_diff>

<commit_message>
Updated test schedule and added highlights
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -768,7 +768,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -871,10 +871,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -5189,16 +5185,16 @@
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9"/>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="27" t="s">
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="13" t="s">
         <v>142</v>
       </c>
@@ -5214,11 +5210,11 @@
       </c>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="R4" s="28"/>
-      <c r="S4" s="28"/>
+      <c r="R4" s="27"/>
+      <c r="S4" s="27"/>
       <c r="T4" s="12" t="s">
         <v>145</v>
       </c>
@@ -5229,22 +5225,22 @@
       </c>
       <c r="X4" s="13"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="27" t="s">
+      <c r="Z4" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="AA4" s="27"/>
-      <c r="AB4" s="27"/>
+      <c r="AA4" s="26"/>
+      <c r="AB4" s="26"/>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="29"/>
-      <c r="E5" s="30" t="s">
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
       <c r="H5" s="13" t="s">
         <v>149</v>
       </c>
@@ -5260,11 +5256,11 @@
       </c>
       <c r="O5" s="17"/>
       <c r="P5" s="17"/>
-      <c r="Q5" s="31" t="s">
+      <c r="Q5" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="R5" s="31"/>
-      <c r="S5" s="31"/>
+      <c r="R5" s="30"/>
+      <c r="S5" s="30"/>
       <c r="T5" s="13" t="s">
         <v>152</v>
       </c>
@@ -5275,17 +5271,17 @@
       </c>
       <c r="X5" s="17"/>
       <c r="Y5" s="17"/>
-      <c r="Z5" s="30" t="s">
+      <c r="Z5" s="29" t="s">
         <v>154</v>
       </c>
-      <c r="AA5" s="30"/>
-      <c r="AB5" s="30"/>
+      <c r="AA5" s="29"/>
+      <c r="AB5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
       <c r="E6" s="17" t="s">
         <v>155</v>
       </c>
@@ -5306,21 +5302,21 @@
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
-      <c r="Q6" s="31" t="s">
+      <c r="Q6" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="R6" s="31"/>
-      <c r="S6" s="31"/>
+      <c r="R6" s="30"/>
+      <c r="S6" s="30"/>
       <c r="T6" s="13" t="s">
         <v>159</v>
       </c>
       <c r="U6" s="13"/>
       <c r="V6" s="13"/>
-      <c r="W6" s="32" t="s">
+      <c r="W6" s="31" t="s">
         <v>159</v>
       </c>
-      <c r="X6" s="32"/>
-      <c r="Y6" s="32"/>
+      <c r="X6" s="31"/>
+      <c r="Y6" s="31"/>
       <c r="Z6" s="17" t="s">
         <v>154</v>
       </c>
@@ -5329,9 +5325,9 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
-      <c r="B7" s="29"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="29"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
       <c r="E7" s="17" t="s">
         <v>160</v>
       </c>
@@ -5352,11 +5348,11 @@
       </c>
       <c r="O7" s="17"/>
       <c r="P7" s="17"/>
-      <c r="Q7" s="31" t="s">
+      <c r="Q7" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="R7" s="31"/>
-      <c r="S7" s="31"/>
+      <c r="R7" s="30"/>
+      <c r="S7" s="30"/>
       <c r="T7" s="13" t="s">
         <v>164</v>
       </c>
@@ -5375,9 +5371,9 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
       <c r="E8" s="17" t="s">
         <v>166</v>
       </c>

</xml_diff>

<commit_message>
Updated tests and added network highlights
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -613,7 +613,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -635,12 +635,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF38"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF38"/>
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
@@ -782,7 +776,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -891,11 +885,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -903,7 +893,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -948,7 +938,7 @@
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF38"/>
+      <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF800000"/>
@@ -5214,21 +5204,21 @@
       </c>
       <c r="I4" s="13"/>
       <c r="J4" s="13"/>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
       <c r="N4" s="13" t="s">
         <v>144</v>
       </c>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
-      <c r="Q4" s="27" t="s">
+      <c r="Q4" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="26"/>
       <c r="T4" s="12" t="s">
         <v>146</v>
       </c>
@@ -5247,14 +5237,14 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29" t="s">
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="28" t="s">
         <v>149</v>
       </c>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
       <c r="H5" s="13" t="s">
         <v>150</v>
       </c>
@@ -5270,21 +5260,21 @@
       </c>
       <c r="O5" s="17"/>
       <c r="P5" s="17"/>
-      <c r="Q5" s="30" t="s">
+      <c r="Q5" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="R5" s="30"/>
-      <c r="S5" s="30"/>
+      <c r="R5" s="29"/>
+      <c r="S5" s="29"/>
       <c r="T5" s="13" t="s">
         <v>154</v>
       </c>
       <c r="U5" s="13"/>
       <c r="V5" s="13"/>
-      <c r="W5" s="17" t="s">
+      <c r="W5" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="X5" s="17"/>
-      <c r="Y5" s="17"/>
+      <c r="X5" s="28"/>
+      <c r="Y5" s="28"/>
       <c r="Z5" s="16" t="s">
         <v>156</v>
       </c>
@@ -5293,9 +5283,9 @@
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
       <c r="E6" s="17" t="s">
         <v>157</v>
       </c>
@@ -5316,32 +5306,32 @@
       </c>
       <c r="O6" s="17"/>
       <c r="P6" s="17"/>
-      <c r="Q6" s="30" t="s">
+      <c r="Q6" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="R6" s="30"/>
-      <c r="S6" s="30"/>
+      <c r="R6" s="29"/>
+      <c r="S6" s="29"/>
       <c r="T6" s="13" t="s">
         <v>161</v>
       </c>
       <c r="U6" s="13"/>
       <c r="V6" s="13"/>
-      <c r="W6" s="31" t="s">
+      <c r="W6" s="30" t="s">
         <v>161</v>
       </c>
-      <c r="X6" s="31"/>
-      <c r="Y6" s="31"/>
-      <c r="Z6" s="17" t="s">
+      <c r="X6" s="30"/>
+      <c r="Y6" s="30"/>
+      <c r="Z6" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="AA6" s="17"/>
-      <c r="AB6" s="17"/>
+      <c r="AA6" s="28"/>
+      <c r="AB6" s="28"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
       <c r="E7" s="17" t="s">
         <v>162</v>
       </c>
@@ -5362,11 +5352,11 @@
       </c>
       <c r="O7" s="17"/>
       <c r="P7" s="17"/>
-      <c r="Q7" s="30" t="s">
+      <c r="Q7" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="R7" s="30"/>
-      <c r="S7" s="30"/>
+      <c r="R7" s="29"/>
+      <c r="S7" s="29"/>
       <c r="T7" s="13" t="s">
         <v>166</v>
       </c>
@@ -5385,9 +5375,9 @@
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
       <c r="E8" s="17" t="s">
         <v>168</v>
       </c>

</xml_diff>

<commit_message>
Added test dates. Added highlights
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -1423,11 +1423,11 @@
       <c r="A7" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
       <c r="E7" s="18" t="s">
         <v>39</v>
       </c>
@@ -5199,21 +5199,21 @@
       </c>
       <c r="F4" s="26"/>
       <c r="G4" s="26"/>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="12" t="s">
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="L4" s="12"/>
-      <c r="M4" s="12"/>
-      <c r="N4" s="13" t="s">
+      <c r="L4" s="26"/>
+      <c r="M4" s="26"/>
+      <c r="N4" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
       <c r="Q4" s="26" t="s">
         <v>145</v>
       </c>
@@ -5321,11 +5321,11 @@
       </c>
       <c r="X6" s="30"/>
       <c r="Y6" s="30"/>
-      <c r="Z6" s="28" t="s">
+      <c r="Z6" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AA6" s="28"/>
-      <c r="AB6" s="28"/>
+      <c r="AA6" s="18"/>
+      <c r="AB6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>

</xml_diff>

<commit_message>
Added new tests. Added maths homework assignment.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5224,11 +5224,11 @@
       </c>
       <c r="U4" s="12"/>
       <c r="V4" s="12"/>
-      <c r="W4" s="13" t="s">
+      <c r="W4" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="X4" s="13"/>
-      <c r="Y4" s="13"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
       <c r="Z4" s="26" t="s">
         <v>148</v>
       </c>
@@ -5286,11 +5286,11 @@
       <c r="B6" s="27"/>
       <c r="C6" s="27"/>
       <c r="D6" s="27"/>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
       <c r="H6" s="13" t="s">
         <v>158</v>
       </c>
@@ -5332,11 +5332,11 @@
       <c r="B7" s="27"/>
       <c r="C7" s="27"/>
       <c r="D7" s="27"/>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
       <c r="H7" s="13" t="s">
         <v>163</v>
       </c>

</xml_diff>

<commit_message>
Added new test dates. Added highlights
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="171">
   <si>
     <t xml:space="preserve">Subject Code</t>
   </si>
@@ -487,6 +487,10 @@
   <si>
     <t xml:space="preserve">Quiz
 Monday 25 May 23:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quiz
+Wednesday 10 June 11:00</t>
   </si>
   <si>
     <t xml:space="preserve">Quiz
@@ -640,14 +644,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FF993300"/>
+        <fgColor theme="7" tint="0.5998"/>
+        <bgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.5998"/>
-        <bgColor rgb="FFFFCC99"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FF993300"/>
       </patternFill>
     </fill>
   </fills>
@@ -776,7 +780,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -885,7 +889,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -893,7 +897,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5237,149 +5245,151 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14"/>
-      <c r="B5" s="27"/>
+      <c r="B5" s="27" t="s">
+        <v>149</v>
+      </c>
       <c r="C5" s="27"/>
       <c r="D5" s="27"/>
       <c r="E5" s="28" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F5" s="28"/>
       <c r="G5" s="28"/>
       <c r="H5" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
       <c r="K5" s="17" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
-      <c r="N5" s="17" t="s">
-        <v>152</v>
-      </c>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
+      <c r="N5" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
       <c r="Q5" s="29" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="R5" s="29"/>
       <c r="S5" s="29"/>
       <c r="T5" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="U5" s="13"/>
       <c r="V5" s="13"/>
       <c r="W5" s="28" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="X5" s="28"/>
       <c r="Y5" s="28"/>
       <c r="Z5" s="16" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA5" s="16"/>
       <c r="AB5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
       <c r="E6" s="28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F6" s="28"/>
       <c r="G6" s="28"/>
       <c r="H6" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
       <c r="K6" s="17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
-      <c r="N6" s="17" t="s">
-        <v>160</v>
-      </c>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
+      <c r="N6" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
       <c r="Q6" s="29" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="R6" s="29"/>
       <c r="S6" s="29"/>
       <c r="T6" s="13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="U6" s="13"/>
       <c r="V6" s="13"/>
-      <c r="W6" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="X6" s="30"/>
-      <c r="Y6" s="30"/>
+      <c r="W6" s="31" t="s">
+        <v>162</v>
+      </c>
+      <c r="X6" s="31"/>
+      <c r="Y6" s="31"/>
       <c r="Z6" s="18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA6" s="18"/>
       <c r="AB6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
       <c r="E7" s="28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F7" s="28"/>
       <c r="G7" s="28"/>
       <c r="H7" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13"/>
       <c r="K7" s="17" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L7" s="17"/>
       <c r="M7" s="17"/>
       <c r="N7" s="17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O7" s="17"/>
       <c r="P7" s="17"/>
       <c r="Q7" s="29" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="R7" s="29"/>
       <c r="S7" s="29"/>
       <c r="T7" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="U7" s="13"/>
       <c r="V7" s="13"/>
       <c r="W7" s="17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="X7" s="17"/>
       <c r="Y7" s="17"/>
       <c r="Z7" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA7" s="17"/>
       <c r="AB7" s="17"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
       <c r="E8" s="17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F8" s="17"/>
       <c r="G8" s="17"/>
@@ -5396,7 +5406,7 @@
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
       <c r="T8" s="17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U8" s="17"/>
       <c r="V8" s="17"/>
@@ -5404,7 +5414,7 @@
       <c r="X8" s="17"/>
       <c r="Y8" s="17"/>
       <c r="Z8" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA8" s="17"/>
       <c r="AB8" s="17"/>
@@ -5436,7 +5446,7 @@
       <c r="X9" s="17"/>
       <c r="Y9" s="17"/>
       <c r="Z9" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA9" s="17"/>
       <c r="AB9" s="17"/>
@@ -5468,7 +5478,7 @@
       <c r="X10" s="17"/>
       <c r="Y10" s="17"/>
       <c r="Z10" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA10" s="17"/>
       <c r="AB10" s="17"/>
@@ -5500,7 +5510,7 @@
       <c r="X11" s="17"/>
       <c r="Y11" s="17"/>
       <c r="Z11" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AA11" s="17"/>
       <c r="AB11" s="17"/>

</xml_diff>

<commit_message>
Added highlight, add new test
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5251,11 +5251,11 @@
       </c>
       <c r="F5" s="28"/>
       <c r="G5" s="28"/>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
       <c r="K5" s="28" t="s">
         <v>151</v>
       </c>

</xml_diff>

<commit_message>
Added highlights and additional tests.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="171">
   <si>
     <t xml:space="preserve">Subject Code</t>
   </si>
@@ -519,6 +519,10 @@
   <si>
     <t xml:space="preserve">Quiz
 Monday 14 Sept 09:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quiz
+Wednesday 8 July 11:00</t>
   </si>
   <si>
     <t xml:space="preserve">Quiz
@@ -885,10 +889,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -897,11 +897,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5241,36 +5245,36 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14"/>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="28" t="s">
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
       <c r="H5" s="12" t="s">
         <v>150</v>
       </c>
       <c r="I5" s="12"/>
       <c r="J5" s="12"/>
-      <c r="K5" s="28" t="s">
+      <c r="K5" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28" t="s">
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="27" t="s">
         <v>152</v>
       </c>
-      <c r="O5" s="28"/>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="29" t="s">
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="28" t="s">
         <v>153</v>
       </c>
-      <c r="R5" s="29"/>
-      <c r="S5" s="29"/>
+      <c r="R5" s="28"/>
+      <c r="S5" s="28"/>
       <c r="T5" s="12" t="s">
         <v>154</v>
       </c>
@@ -5289,44 +5293,46 @@
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="28" t="s">
+      <c r="B6" s="29" t="s">
         <v>157</v>
       </c>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="27" t="s">
+        <v>158</v>
+      </c>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
       <c r="H6" s="13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
       <c r="K6" s="17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="L6" s="17"/>
       <c r="M6" s="17"/>
-      <c r="N6" s="28" t="s">
-        <v>160</v>
-      </c>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="R6" s="29"/>
-      <c r="S6" s="29"/>
+      <c r="N6" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
+      <c r="Q6" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="R6" s="28"/>
+      <c r="S6" s="28"/>
       <c r="T6" s="12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="U6" s="12"/>
       <c r="V6" s="12"/>
-      <c r="W6" s="31" t="s">
-        <v>161</v>
-      </c>
-      <c r="X6" s="31"/>
-      <c r="Y6" s="31"/>
+      <c r="W6" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="X6" s="30"/>
+      <c r="Y6" s="30"/>
       <c r="Z6" s="18" t="s">
         <v>156</v>
       </c>
@@ -5335,57 +5341,57 @@
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="27" t="s">
+        <v>163</v>
+      </c>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
       <c r="H7" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="13"/>
       <c r="K7" s="17" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="L7" s="17"/>
       <c r="M7" s="17"/>
       <c r="N7" s="17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O7" s="17"/>
       <c r="P7" s="17"/>
-      <c r="Q7" s="29" t="s">
-        <v>165</v>
-      </c>
-      <c r="R7" s="29"/>
-      <c r="S7" s="29"/>
-      <c r="T7" s="13" t="s">
+      <c r="Q7" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="U7" s="12"/>
+      <c r="V7" s="12"/>
       <c r="W7" s="17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="X7" s="17"/>
       <c r="Y7" s="17"/>
-      <c r="Z7" s="28" t="s">
+      <c r="Z7" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="AA7" s="28"/>
-      <c r="AB7" s="28"/>
+      <c r="AA7" s="27"/>
+      <c r="AB7" s="27"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
       <c r="E8" s="17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F8" s="17"/>
       <c r="G8" s="17"/>
@@ -5402,18 +5408,18 @@
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
       <c r="T8" s="17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="U8" s="17"/>
       <c r="V8" s="17"/>
       <c r="W8" s="17"/>
       <c r="X8" s="17"/>
       <c r="Y8" s="17"/>
-      <c r="Z8" s="17" t="s">
+      <c r="Z8" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="AA8" s="17"/>
-      <c r="AB8" s="17"/>
+      <c r="AA8" s="27"/>
+      <c r="AB8" s="27"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14"/>

</xml_diff>

<commit_message>
Added new test finished
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -893,11 +893,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5265,16 +5265,16 @@
       </c>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
-      <c r="N5" s="27" t="s">
+      <c r="N5" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="28" t="s">
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="27" t="s">
         <v>153</v>
       </c>
-      <c r="R5" s="28"/>
-      <c r="S5" s="28"/>
+      <c r="R5" s="27"/>
+      <c r="S5" s="27"/>
       <c r="T5" s="12" t="s">
         <v>154</v>
       </c>
@@ -5293,11 +5293,11 @@
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="28" t="s">
         <v>157</v>
       </c>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
       <c r="E6" s="27" t="s">
         <v>158</v>
       </c>
@@ -5318,11 +5318,11 @@
       </c>
       <c r="O6" s="27"/>
       <c r="P6" s="27"/>
-      <c r="Q6" s="28" t="s">
+      <c r="Q6" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="R6" s="28"/>
-      <c r="S6" s="28"/>
+      <c r="R6" s="29"/>
+      <c r="S6" s="29"/>
       <c r="T6" s="12" t="s">
         <v>162</v>
       </c>
@@ -5364,11 +5364,11 @@
       </c>
       <c r="O7" s="17"/>
       <c r="P7" s="17"/>
-      <c r="Q7" s="28" t="s">
+      <c r="Q7" s="29" t="s">
         <v>166</v>
       </c>
-      <c r="R7" s="28"/>
-      <c r="S7" s="28"/>
+      <c r="R7" s="29"/>
+      <c r="S7" s="29"/>
       <c r="T7" s="12" t="s">
         <v>167</v>
       </c>

</xml_diff>

<commit_message>
Added additional docs. Finished test.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5275,11 +5275,11 @@
       </c>
       <c r="R5" s="27"/>
       <c r="S5" s="27"/>
-      <c r="T5" s="12" t="s">
+      <c r="T5" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="U5" s="12"/>
-      <c r="V5" s="12"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="26"/>
       <c r="W5" s="18" t="s">
         <v>155</v>
       </c>

</xml_diff>

<commit_message>
Added new assignment question. Finished assignment
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5282,11 +5282,11 @@
       </c>
       <c r="O5" s="18"/>
       <c r="P5" s="18"/>
-      <c r="Q5" s="27" t="s">
+      <c r="Q5" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
       <c r="T5" s="26" t="s">
         <v>154</v>
       </c>

</xml_diff>

<commit_message>
Added highlights and tests.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5404,11 +5404,11 @@
       <c r="B8" s="31"/>
       <c r="C8" s="31"/>
       <c r="D8" s="31"/>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="27" t="s">
         <v>172</v>
       </c>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
       <c r="J8" s="17"/>

</xml_diff>

<commit_message>
Finished assessment, marked done.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -685,7 +685,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -714,6 +714,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFAFD095"/>
         <bgColor rgb="FF99CCFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF860D"/>
+        <bgColor rgb="FFFF6600"/>
       </patternFill>
     </fill>
   </fills>
@@ -963,11 +969,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1026,7 +1032,7 @@
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF860D"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
@@ -5413,11 +5419,11 @@
       </c>
       <c r="F7" s="18"/>
       <c r="G7" s="18"/>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="26" t="s">
         <v>167</v>
       </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
       <c r="K7" s="17" t="s">
         <v>168</v>
       </c>
@@ -5433,11 +5439,11 @@
       </c>
       <c r="R7" s="29"/>
       <c r="S7" s="29"/>
-      <c r="T7" s="12" t="s">
+      <c r="T7" s="26" t="s">
         <v>171</v>
       </c>
-      <c r="U7" s="12"/>
-      <c r="V7" s="12"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26"/>
       <c r="W7" s="29" t="s">
         <v>172</v>
       </c>

</xml_diff>

<commit_message>
Added textbook. Marked tests done.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5449,11 +5449,11 @@
       </c>
       <c r="X7" s="29"/>
       <c r="Y7" s="29"/>
-      <c r="Z7" s="29" t="s">
+      <c r="Z7" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AA7" s="29"/>
-      <c r="AB7" s="29"/>
+      <c r="AA7" s="18"/>
+      <c r="AB7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
@@ -5462,11 +5462,11 @@
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
-      <c r="E8" s="29" t="s">
+      <c r="E8" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
       <c r="J8" s="17"/>
@@ -5479,19 +5479,19 @@
       <c r="Q8" s="17"/>
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
-      <c r="T8" s="29" t="s">
+      <c r="T8" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="U8" s="29"/>
-      <c r="V8" s="29"/>
+      <c r="U8" s="27"/>
+      <c r="V8" s="27"/>
       <c r="W8" s="17"/>
       <c r="X8" s="17"/>
       <c r="Y8" s="17"/>
-      <c r="Z8" s="29" t="s">
+      <c r="Z8" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AA8" s="29"/>
-      <c r="AB8" s="29"/>
+      <c r="AA8" s="18"/>
+      <c r="AB8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14"/>
@@ -5519,11 +5519,11 @@
       <c r="W9" s="17"/>
       <c r="X9" s="17"/>
       <c r="Y9" s="17"/>
-      <c r="Z9" s="29" t="s">
+      <c r="Z9" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AA9" s="29"/>
-      <c r="AB9" s="29"/>
+      <c r="AA9" s="18"/>
+      <c r="AB9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14"/>
@@ -5551,11 +5551,11 @@
       <c r="W10" s="17"/>
       <c r="X10" s="17"/>
       <c r="Y10" s="17"/>
-      <c r="Z10" s="29" t="s">
+      <c r="Z10" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AA10" s="29"/>
-      <c r="AB10" s="29"/>
+      <c r="AA10" s="18"/>
+      <c r="AB10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>

</xml_diff>

<commit_message>
Marked assignment as done.
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -957,15 +957,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5386,21 +5386,21 @@
       </c>
       <c r="O6" s="18"/>
       <c r="P6" s="18"/>
-      <c r="Q6" s="27" t="s">
+      <c r="Q6" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="R6" s="27"/>
-      <c r="S6" s="27"/>
+      <c r="R6" s="18"/>
+      <c r="S6" s="18"/>
       <c r="T6" s="26" t="s">
         <v>163</v>
       </c>
       <c r="U6" s="26"/>
       <c r="V6" s="26"/>
-      <c r="W6" s="28" t="s">
+      <c r="W6" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="X6" s="28"/>
-      <c r="Y6" s="28"/>
+      <c r="X6" s="27"/>
+      <c r="Y6" s="27"/>
       <c r="Z6" s="18" t="s">
         <v>156</v>
       </c>
@@ -5429,26 +5429,26 @@
       </c>
       <c r="L7" s="17"/>
       <c r="M7" s="17"/>
-      <c r="N7" s="29" t="s">
+      <c r="N7" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="O7" s="29"/>
-      <c r="P7" s="29"/>
-      <c r="Q7" s="29" t="s">
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="R7" s="29"/>
-      <c r="S7" s="29"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28"/>
       <c r="T7" s="26" t="s">
         <v>171</v>
       </c>
       <c r="U7" s="26"/>
       <c r="V7" s="26"/>
-      <c r="W7" s="29" t="s">
+      <c r="W7" s="28" t="s">
         <v>172</v>
       </c>
-      <c r="X7" s="29"/>
-      <c r="Y7" s="29"/>
+      <c r="X7" s="28"/>
+      <c r="Y7" s="28"/>
       <c r="Z7" s="18" t="s">
         <v>156</v>
       </c>
@@ -5479,11 +5479,11 @@
       <c r="Q8" s="17"/>
       <c r="R8" s="17"/>
       <c r="S8" s="17"/>
-      <c r="T8" s="27" t="s">
+      <c r="T8" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="U8" s="27"/>
-      <c r="V8" s="27"/>
+      <c r="U8" s="29"/>
+      <c r="V8" s="29"/>
       <c r="W8" s="17"/>
       <c r="X8" s="17"/>
       <c r="Y8" s="17"/>
@@ -5583,11 +5583,11 @@
       <c r="W11" s="17"/>
       <c r="X11" s="17"/>
       <c r="Y11" s="17"/>
-      <c r="Z11" s="29" t="s">
+      <c r="Z11" s="28" t="s">
         <v>156</v>
       </c>
-      <c r="AA11" s="29"/>
-      <c r="AB11" s="29"/>
+      <c r="AA11" s="28"/>
+      <c r="AB11" s="28"/>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>

</xml_diff>

<commit_message>
Marked test as done
</commit_message>
<xml_diff>
--- a/curriculum.xlsx
+++ b/curriculum.xlsx
@@ -5429,11 +5429,11 @@
       </c>
       <c r="L7" s="17"/>
       <c r="M7" s="17"/>
-      <c r="N7" s="28" t="s">
+      <c r="N7" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="O7" s="28"/>
-      <c r="P7" s="28"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
       <c r="Q7" s="28" t="s">
         <v>170</v>
       </c>
@@ -5583,11 +5583,11 @@
       <c r="W11" s="17"/>
       <c r="X11" s="17"/>
       <c r="Y11" s="17"/>
-      <c r="Z11" s="28" t="s">
+      <c r="Z11" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="AA11" s="28"/>
-      <c r="AB11" s="28"/>
+      <c r="AA11" s="18"/>
+      <c r="AB11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>

</xml_diff>